<commit_message>
Halfway through the tests
</commit_message>
<xml_diff>
--- a/tests/features/assets/valid_minimal.xlsx
+++ b/tests/features/assets/valid_minimal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrique/PycharmProjects/biobroker/tests/features/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C60543-8D7C-764B-96AB-4CA8937E0AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{402B9E3E-05D1-FA45-BFAC-01B14A3BD425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="34560" windowHeight="22340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -116,7 +116,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>

</xml_diff>